<commit_message>
Final ST accruals :D
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/BMAX.ST.xlsx
+++ b/data/stx_xlsx/BMAX.ST.xlsx
@@ -9601,7 +9601,9 @@
       <c r="L43" s="21">
         <v>25.12</v>
       </c>
-      <c r="M43" s="20"/>
+      <c r="M43" s="21">
+        <v>29.62</v>
+      </c>
       <c r="N43" s="21">
         <v>23.28</v>
       </c>

</xml_diff>